<commit_message>
Remove Changed By column from Change_Log.xlsx
Drop the Changed By column at the user's request; the log now has 14
columns. Update CLAUDE.md to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/04_Change_Records/Change_Log.xlsx
+++ b/Documentation/04_Change_Records/Change_Log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Change_Log!$A$1:$O$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Change_Log!$A$1:$N$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -51,9 +51,6 @@
     <t>API Name</t>
   </si>
   <si>
-    <t>Changed By</t>
-  </si>
-  <si>
     <t>Reason</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
   </si>
   <si>
     <t>Cases_disposition</t>
-  </si>
-  <si>
-    <t>Raghav (via Claude Code); deployed with Salesforce CLI signed in as Sandip Patel's user</t>
   </si>
   <si>
     <t>To align the Sandbox Case Disposition Flow with the Production configuration.</t>
@@ -1387,7 +1381,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="12.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="12.6363636363636" style="4" customWidth="1"/>
@@ -1395,18 +1389,17 @@
     <col min="3" max="3" width="14.6363636363636" style="2" customWidth="1"/>
     <col min="4" max="4" width="18.6363636363636" style="2" customWidth="1"/>
     <col min="5" max="6" width="20.6363636363636" style="2" customWidth="1"/>
-    <col min="7" max="7" width="26.6363636363636" style="2" customWidth="1"/>
-    <col min="8" max="8" width="32.6363636363636" style="2" customWidth="1"/>
-    <col min="9" max="9" width="48.6363636363636" style="2" customWidth="1"/>
-    <col min="10" max="10" width="52.6363636363636" style="2" customWidth="1"/>
-    <col min="11" max="11" width="44.6363636363636" style="2" customWidth="1"/>
-    <col min="12" max="12" width="40.6363636363636" style="2" customWidth="1"/>
-    <col min="13" max="14" width="34.6363636363636" style="2" customWidth="1"/>
-    <col min="15" max="15" width="44.6363636363636" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="8.72727272727273" style="2"/>
+    <col min="7" max="7" width="32.6363636363636" style="2" customWidth="1"/>
+    <col min="8" max="8" width="48.6363636363636" style="2" customWidth="1"/>
+    <col min="9" max="9" width="52.6363636363636" style="2" customWidth="1"/>
+    <col min="10" max="10" width="44.6363636363636" style="2" customWidth="1"/>
+    <col min="11" max="11" width="40.6363636363636" style="2" customWidth="1"/>
+    <col min="12" max="13" width="34.6363636363636" style="2" customWidth="1"/>
+    <col min="14" max="14" width="44.6363636363636" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.72727272727273" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:15">
+    <row r="1" ht="30" customHeight="1" spans="1:14">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1449,111 +1442,102 @@
       <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+    </row>
+    <row r="2" ht="58" spans="1:14">
+      <c r="A2" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="B2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" ht="58" spans="1:15">
-      <c r="A2" s="7" t="s">
+    <row r="3" ht="62.5" spans="1:14">
+      <c r="A3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="8" t="s">
+      <c r="G3" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="H3" s="8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" ht="62.5" spans="1:15">
-      <c r="A3" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="N3" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:O3" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N3" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="O2" r:id="rId1" display="https://teamvelocity--fullsando.sandbox.my.salesforce.com/builder_platform_interaction/flowBuilder.app?flowId=301Va000015R2iVIAS" tooltip="Open in Flow Builder"/>
-    <hyperlink ref="O3" r:id="rId2" display="https://teamvelocity--fullsando.sandbox.my.salesforce.com/builder_platform_interaction/flowBuilder.app?flowId=301Va000015RMAjIAO" tooltip="Open in Flow Builder"/>
+    <hyperlink ref="N2" r:id="rId1" display="https://teamvelocity--fullsando.sandbox.my.salesforce.com/builder_platform_interaction/flowBuilder.app?flowId=301Va000015R2iVIAS" tooltip="Open in Flow Builder"/>
+    <hyperlink ref="N3" r:id="rId2" display="https://teamvelocity--fullsando.sandbox.my.salesforce.com/builder_platform_interaction/flowBuilder.app?flowId=301Va000015RMAjIAO" tooltip="Open in Flow Builder"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1572,52 +1556,52 @@
   <sheetData>
     <row r="1" ht="15.5" spans="1:1">
       <c r="A1" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" ht="25" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>